<commit_message>
verificación datos 2025 y 2026
</commit_message>
<xml_diff>
--- a/salidas/Base_resultados_PPDJ_python.xlsx
+++ b/salidas/Base_resultados_PPDJ_python.xlsx
@@ -719,55 +719,55 @@
         <v>0.44</v>
       </c>
       <c r="L3" t="n">
-        <v>0.32</v>
+        <v>0.323</v>
       </c>
       <c r="M3" t="n">
-        <v>0.12</v>
+        <v>0.117</v>
       </c>
       <c r="N3" t="n">
         <v>0.44</v>
       </c>
       <c r="O3" t="n">
-        <v>0.33</v>
+        <v>0.333</v>
       </c>
       <c r="P3" t="n">
-        <v>0.11</v>
+        <v>0.107</v>
       </c>
       <c r="Q3" t="n">
         <v>0.34</v>
       </c>
       <c r="R3" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="S3" t="n">
-        <v>-0</v>
+        <v>-0.003</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.35</v>
+        <v>0.353</v>
       </c>
       <c r="V3" t="n">
-        <v>-0.35</v>
+        <v>-0.353</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>0.36</v>
+        <v>0.363</v>
       </c>
       <c r="Y3" t="n">
-        <v>-0.36</v>
+        <v>-0.363</v>
       </c>
       <c r="Z3" t="n">
         <v>0.34</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.37</v>
+        <v>0.373</v>
       </c>
       <c r="AB3" t="n">
-        <v>-0.03</v>
+        <v>-0.033</v>
       </c>
     </row>
     <row r="4">
@@ -832,28 +832,28 @@
         <v>0.1</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="P4" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.1</v>
+        <v>-0.105</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="V4" t="n">
-        <v>-0.1</v>
+        <v>-0.105</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
@@ -933,13 +933,13 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.01</v>
+        <v>0.0119</v>
       </c>
       <c r="O5" t="n">
         <v>5</v>
       </c>
       <c r="P5" t="n">
-        <v>-4.99</v>
+        <v>-4.9881</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -1027,55 +1027,55 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.92</v>
+        <v>-0.924</v>
       </c>
       <c r="N6" t="n">
-        <v>0.01</v>
+        <v>0.0102</v>
       </c>
       <c r="O6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.91</v>
+        <v>-0.9137999999999999</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.11</v>
+        <v>1.106</v>
       </c>
       <c r="R6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="S6" t="n">
-        <v>0.18</v>
+        <v>0.182</v>
       </c>
       <c r="T6" t="n">
-        <v>1.04</v>
+        <v>1.0385</v>
       </c>
       <c r="U6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="V6" t="n">
-        <v>0.11</v>
+        <v>0.1145</v>
       </c>
       <c r="W6" t="n">
         <v>100.58</v>
       </c>
       <c r="X6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="Y6" t="n">
-        <v>99.66</v>
+        <v>99.65600000000001</v>
       </c>
       <c r="Z6" t="n">
         <v>102.02</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.92</v>
+        <v>0.924</v>
       </c>
       <c r="AB6" t="n">
-        <v>101.1</v>
+        <v>101.096</v>
       </c>
     </row>
     <row r="7">
@@ -1131,55 +1131,55 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.82</v>
+        <v>-0.823</v>
       </c>
       <c r="N7" t="n">
-        <v>0.01</v>
+        <v>0.0051</v>
       </c>
       <c r="O7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.82</v>
+        <v>-0.8179</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.98</v>
+        <v>0.978</v>
       </c>
       <c r="R7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="S7" t="n">
-        <v>0.16</v>
+        <v>0.155</v>
       </c>
       <c r="T7" t="n">
-        <v>0.99</v>
+        <v>0.9876</v>
       </c>
       <c r="U7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="V7" t="n">
-        <v>0.16</v>
+        <v>0.1646</v>
       </c>
       <c r="W7" t="n">
-        <v>0.98</v>
+        <v>0.9754</v>
       </c>
       <c r="X7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.15</v>
+        <v>0.1524</v>
       </c>
       <c r="Z7" t="n">
         <v>101.79</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.82</v>
+        <v>0.823</v>
       </c>
       <c r="AB7" t="n">
-        <v>100.97</v>
+        <v>100.967</v>
       </c>
     </row>
     <row r="8">
@@ -1235,55 +1235,55 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.5580000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>0.48</v>
+        <v>0.482</v>
       </c>
       <c r="O8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.08</v>
+        <v>-0.076</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.48</v>
+        <v>0.482</v>
       </c>
       <c r="R8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.08</v>
+        <v>-0.081</v>
       </c>
       <c r="T8" t="n">
-        <v>0.52</v>
+        <v>0.515</v>
       </c>
       <c r="U8" t="n">
-        <v>0.57</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.05</v>
+        <v>-0.053</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0.57</v>
+        <v>0.573</v>
       </c>
       <c r="Y8" t="n">
-        <v>-0.57</v>
+        <v>-0.573</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.54</v>
+        <v>0.5391</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.58</v>
+        <v>0.578</v>
       </c>
       <c r="AB8" t="n">
-        <v>-0.04</v>
+        <v>-0.0389</v>
       </c>
     </row>
     <row r="9">
@@ -1372,13 +1372,13 @@
         <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>1</v>
+        <v>0.9991</v>
       </c>
       <c r="X9" t="n">
         <v>1</v>
       </c>
       <c r="Y9" t="n">
-        <v>-0</v>
+        <v>-0.0009</v>
       </c>
       <c r="Z9" t="n">
         <v>1</v>
@@ -1452,37 +1452,37 @@
         <v>0.35</v>
       </c>
       <c r="O10" t="n">
-        <v>0.32</v>
+        <v>0.3216</v>
       </c>
       <c r="P10" t="n">
-        <v>0.03</v>
+        <v>0.0284</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.35</v>
+        <v>0.352</v>
       </c>
       <c r="R10" t="n">
-        <v>0.32</v>
+        <v>0.3216</v>
       </c>
       <c r="S10" t="n">
-        <v>0.03</v>
+        <v>0.0304</v>
       </c>
       <c r="T10" t="n">
         <v>0.35</v>
       </c>
       <c r="U10" t="n">
-        <v>0.32</v>
+        <v>0.3216</v>
       </c>
       <c r="V10" t="n">
-        <v>0.03</v>
+        <v>0.0284</v>
       </c>
       <c r="W10" t="n">
-        <v>0.33</v>
+        <v>0.325</v>
       </c>
       <c r="X10" t="n">
         <v>0.32</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="Z10" t="n">
         <v>0.33</v>
@@ -1562,31 +1562,31 @@
         <v>-0.13</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="R11" t="n">
         <v>1.53</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.52</v>
+        <v>-1.524</v>
       </c>
       <c r="T11" t="n">
-        <v>0.04</v>
+        <v>0.035</v>
       </c>
       <c r="U11" t="n">
         <v>1.53</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.5</v>
+        <v>-1.495</v>
       </c>
       <c r="W11" t="n">
-        <v>0.02</v>
+        <v>0.0216</v>
       </c>
       <c r="X11" t="n">
         <v>1.53</v>
       </c>
       <c r="Y11" t="n">
-        <v>-1.51</v>
+        <v>-1.5084</v>
       </c>
       <c r="Z11" t="n">
         <v>2</v>
@@ -1673,13 +1673,13 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>0.09</v>
+        <v>0.0949</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.09</v>
+        <v>0.0906</v>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>0.0043</v>
       </c>
     </row>
     <row r="13">
@@ -1741,31 +1741,31 @@
         <v>0.37</v>
       </c>
       <c r="N13" t="n">
-        <v>0.25</v>
+        <v>0.251</v>
       </c>
       <c r="O13" t="n">
         <v>0.27</v>
       </c>
       <c r="P13" t="n">
-        <v>-0.02</v>
+        <v>-0.019</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.91</v>
+        <v>0.9079</v>
       </c>
       <c r="R13" t="n">
         <v>0.28</v>
       </c>
       <c r="S13" t="n">
-        <v>0.63</v>
+        <v>0.6279</v>
       </c>
       <c r="T13" t="n">
-        <v>0.31</v>
+        <v>0.3085</v>
       </c>
       <c r="U13" t="n">
         <v>0.3</v>
       </c>
       <c r="V13" t="n">
-        <v>0.01</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="W13" t="n">
         <v>0.5</v>
@@ -1863,22 +1863,22 @@
         <v>-0.27</v>
       </c>
       <c r="T14" t="n">
-        <v>0.11</v>
+        <v>0.1053</v>
       </c>
       <c r="U14" t="n">
         <v>0.4</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.29</v>
+        <v>-0.2947</v>
       </c>
       <c r="W14" t="n">
-        <v>0.17</v>
+        <v>0.172</v>
       </c>
       <c r="X14" t="n">
         <v>0.4</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.23</v>
+        <v>-0.228</v>
       </c>
       <c r="Z14" t="n">
         <v>0.16</v>
@@ -1940,58 +1940,58 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>0.28</v>
+        <v>0.2771</v>
       </c>
       <c r="L15" t="n">
-        <v>0.23</v>
+        <v>0.233</v>
       </c>
       <c r="M15" t="n">
-        <v>0.04</v>
+        <v>0.0441</v>
       </c>
       <c r="N15" t="n">
         <v>4.94</v>
       </c>
       <c r="O15" t="n">
-        <v>0.25</v>
+        <v>0.252</v>
       </c>
       <c r="P15" t="n">
-        <v>4.69</v>
+        <v>4.688</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.36</v>
+        <v>0.3625</v>
       </c>
       <c r="R15" t="n">
-        <v>0.27</v>
+        <v>0.2663</v>
       </c>
       <c r="S15" t="n">
-        <v>0.1</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="T15" t="n">
-        <v>0.36</v>
+        <v>0.3626</v>
       </c>
       <c r="U15" t="n">
-        <v>0.28</v>
+        <v>0.2762</v>
       </c>
       <c r="V15" t="n">
-        <v>0.09</v>
+        <v>0.0864</v>
       </c>
       <c r="W15" t="n">
-        <v>0.36</v>
+        <v>0.3626</v>
       </c>
       <c r="X15" t="n">
-        <v>0.29</v>
+        <v>0.2885</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.0741</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.36</v>
+        <v>0.3626</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.3</v>
+        <v>0.3008</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.06</v>
+        <v>0.0618</v>
       </c>
     </row>
     <row r="16">
@@ -2261,22 +2261,22 @@
         <v>27.16</v>
       </c>
       <c r="N18" t="n">
-        <v>0.3</v>
+        <v>0.3005</v>
       </c>
       <c r="O18" t="n">
         <v>34.6</v>
       </c>
       <c r="P18" t="n">
-        <v>-34.3</v>
+        <v>-34.2995</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.22</v>
+        <v>0.2195</v>
       </c>
       <c r="R18" t="n">
         <v>32.8</v>
       </c>
       <c r="S18" t="n">
-        <v>-32.58</v>
+        <v>-32.5805</v>
       </c>
       <c r="T18" t="n">
         <v>41.4</v>
@@ -2472,46 +2472,46 @@
         <v>0.2</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1</v>
+        <v>0.104</v>
       </c>
       <c r="P20" t="n">
-        <v>0.1</v>
+        <v>0.096</v>
       </c>
       <c r="Q20" t="n">
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>0.11</v>
+        <v>0.114</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.11</v>
+        <v>-0.114</v>
       </c>
       <c r="T20" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="U20" t="n">
-        <v>0.12</v>
+        <v>0.124</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.09</v>
+        <v>-0.091</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.0675</v>
       </c>
       <c r="X20" t="n">
-        <v>0.12</v>
+        <v>0.124</v>
       </c>
       <c r="Y20" t="n">
-        <v>-0.06</v>
+        <v>-0.0565</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.0675</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.13</v>
+        <v>0.134</v>
       </c>
       <c r="AB20" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.0665</v>
       </c>
     </row>
     <row r="21">
@@ -2567,55 +2567,55 @@
         <v>0.18</v>
       </c>
       <c r="L21" t="n">
-        <v>0.32</v>
+        <v>0.323</v>
       </c>
       <c r="M21" t="n">
-        <v>-0.14</v>
+        <v>-0.143</v>
       </c>
       <c r="N21" t="n">
         <v>0.18</v>
       </c>
       <c r="O21" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="P21" t="n">
-        <v>-0.16</v>
+        <v>-0.163</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>0.36</v>
+        <v>0.363</v>
       </c>
       <c r="S21" t="n">
-        <v>-0.36</v>
+        <v>-0.363</v>
       </c>
       <c r="T21" t="n">
-        <v>0.14</v>
+        <v>0.144</v>
       </c>
       <c r="U21" t="n">
-        <v>0.38</v>
+        <v>0.383</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.24</v>
+        <v>-0.239</v>
       </c>
       <c r="W21" t="n">
-        <v>0.14</v>
+        <v>0.1353</v>
       </c>
       <c r="X21" t="n">
-        <v>0.38</v>
+        <v>0.383</v>
       </c>
       <c r="Y21" t="n">
-        <v>-0.25</v>
+        <v>-0.2477</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.14</v>
+        <v>0.1353</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.4</v>
+        <v>0.403</v>
       </c>
       <c r="AB21" t="n">
-        <v>-0.27</v>
+        <v>-0.2677</v>
       </c>
     </row>
     <row r="22">
@@ -2686,13 +2686,13 @@
         <v>-3.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="R22" t="n">
         <v>5</v>
       </c>
       <c r="S22" t="n">
-        <v>-4.93</v>
+        <v>-4.932</v>
       </c>
       <c r="T22" t="n">
         <v>6.03</v>
@@ -2808,13 +2808,13 @@
         <v>-0.11</v>
       </c>
       <c r="W23" t="n">
-        <v>0.52</v>
+        <v>0.5165</v>
       </c>
       <c r="X23" t="n">
         <v>0.61</v>
       </c>
       <c r="Y23" t="n">
-        <v>-0.09</v>
+        <v>-0.0935</v>
       </c>
       <c r="Z23" t="n">
         <v>0.52</v>
@@ -3092,28 +3092,28 @@
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>1062.26</v>
+        <v>1062.2569</v>
       </c>
       <c r="P26" t="n">
-        <v>-1062.26</v>
+        <v>-1062.2569</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
       </c>
       <c r="R26" t="n">
-        <v>1045.83</v>
+        <v>1045.8303</v>
       </c>
       <c r="S26" t="n">
-        <v>-1045.83</v>
+        <v>-1045.8303</v>
       </c>
       <c r="T26" t="n">
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>1029.4</v>
+        <v>1029.4036</v>
       </c>
       <c r="V26" t="n">
-        <v>-1029.4</v>
+        <v>-1029.4036</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -3287,55 +3287,55 @@
         <v>0.4</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>0.9999</v>
       </c>
       <c r="M28" t="n">
-        <v>-0.6</v>
+        <v>-0.5999</v>
       </c>
       <c r="N28" t="n">
         <v>0.51</v>
       </c>
       <c r="O28" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="P28" t="n">
-        <v>-0.49</v>
+        <v>-0.4898</v>
       </c>
       <c r="Q28" t="n">
         <v>1.1</v>
       </c>
       <c r="R28" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="S28" t="n">
-        <v>0.1</v>
+        <v>0.1003</v>
       </c>
       <c r="T28" t="n">
         <v>1.62</v>
       </c>
       <c r="U28" t="n">
-        <v>1</v>
+        <v>0.9996</v>
       </c>
       <c r="V28" t="n">
-        <v>0.62</v>
+        <v>0.6204</v>
       </c>
       <c r="W28" t="n">
         <v>0</v>
       </c>
       <c r="X28" t="n">
-        <v>1</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="Y28" t="n">
-        <v>-1</v>
+        <v>-0.9995000000000001</v>
       </c>
       <c r="Z28" t="n">
-        <v>3.06</v>
+        <v>3.0612</v>
       </c>
       <c r="AA28" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="AB28" t="n">
-        <v>2.06</v>
+        <v>2.0618</v>
       </c>
     </row>
     <row r="29">
@@ -3391,55 +3391,55 @@
         <v>0.4</v>
       </c>
       <c r="L29" t="n">
-        <v>0.01</v>
+        <v>0.0109</v>
       </c>
       <c r="M29" t="n">
-        <v>0.39</v>
+        <v>0.3891</v>
       </c>
       <c r="N29" t="n">
         <v>0.82</v>
       </c>
       <c r="O29" t="n">
-        <v>0.01</v>
+        <v>0.0109</v>
       </c>
       <c r="P29" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8091</v>
       </c>
       <c r="Q29" t="n">
         <v>3.04</v>
       </c>
       <c r="R29" t="n">
-        <v>0.01</v>
+        <v>0.0108</v>
       </c>
       <c r="S29" t="n">
-        <v>3.03</v>
+        <v>3.0292</v>
       </c>
       <c r="T29" t="n">
         <v>3.83</v>
       </c>
       <c r="U29" t="n">
-        <v>0.01</v>
+        <v>0.0107</v>
       </c>
       <c r="V29" t="n">
-        <v>3.82</v>
+        <v>3.8193</v>
       </c>
       <c r="W29" t="n">
         <v>0</v>
       </c>
       <c r="X29" t="n">
-        <v>0.01</v>
+        <v>0.0107</v>
       </c>
       <c r="Y29" t="n">
-        <v>-0.01</v>
+        <v>-0.0107</v>
       </c>
       <c r="Z29" t="n">
         <v>4.66</v>
       </c>
       <c r="AA29" t="n">
-        <v>0.01</v>
+        <v>0.0106</v>
       </c>
       <c r="AB29" t="n">
-        <v>4.65</v>
+        <v>4.6494</v>
       </c>
     </row>
     <row r="30">
@@ -3495,50 +3495,50 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0.89</v>
+        <v>0.8863</v>
       </c>
       <c r="M30" t="n">
-        <v>-0.89</v>
+        <v>-0.8863</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>0.88</v>
+        <v>0.8763</v>
       </c>
       <c r="P30" t="n">
-        <v>-0.88</v>
+        <v>-0.8763</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
       </c>
       <c r="R30" t="n">
-        <v>0.87</v>
+        <v>0.8663</v>
       </c>
       <c r="S30" t="n">
-        <v>-0.87</v>
+        <v>-0.8663</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>0.86</v>
+        <v>0.8563</v>
       </c>
       <c r="V30" t="n">
-        <v>-0.86</v>
+        <v>-0.8563</v>
       </c>
       <c r="W30" t="n">
         <v>0</v>
       </c>
       <c r="X30" t="n">
-        <v>0.86</v>
+        <v>0.8563</v>
       </c>
       <c r="Y30" t="n">
-        <v>-0.86</v>
+        <v>-0.8563</v>
       </c>
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="n">
-        <v>0.85</v>
+        <v>0.8463000000000001</v>
       </c>
       <c r="AB30" t="inlineStr"/>
     </row>
@@ -3699,50 +3699,50 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0.19</v>
+        <v>0.1919</v>
       </c>
       <c r="M32" t="n">
-        <v>-0.19</v>
+        <v>-0.1919</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>0.19</v>
+        <v>0.1908</v>
       </c>
       <c r="P32" t="n">
-        <v>-0.19</v>
+        <v>-0.1908</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>0.19</v>
+        <v>0.1897</v>
       </c>
       <c r="S32" t="n">
-        <v>-0.19</v>
+        <v>-0.1897</v>
       </c>
       <c r="T32" t="n">
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>0.19</v>
+        <v>0.1886</v>
       </c>
       <c r="V32" t="n">
-        <v>-0.19</v>
+        <v>-0.1886</v>
       </c>
       <c r="W32" t="n">
         <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>0.19</v>
+        <v>0.1886</v>
       </c>
       <c r="Y32" t="n">
-        <v>-0.19</v>
+        <v>-0.1886</v>
       </c>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="n">
-        <v>0.19</v>
+        <v>0.1875</v>
       </c>
       <c r="AB32" t="inlineStr"/>
     </row>
@@ -3796,58 +3796,58 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>0.1</v>
+        <v>0.1005</v>
       </c>
       <c r="L33" t="n">
-        <v>0.61</v>
+        <v>0.613</v>
       </c>
       <c r="M33" t="n">
-        <v>-0.51</v>
+        <v>-0.5125</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>0.61</v>
+        <v>0.6145</v>
       </c>
       <c r="P33" t="n">
-        <v>-0.61</v>
+        <v>-0.6145</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.25</v>
+        <v>0.2525</v>
       </c>
       <c r="R33" t="n">
-        <v>0.62</v>
+        <v>0.616</v>
       </c>
       <c r="S33" t="n">
-        <v>-0.36</v>
+        <v>-0.3635</v>
       </c>
       <c r="T33" t="n">
         <v>0.98</v>
       </c>
       <c r="U33" t="n">
-        <v>0.62</v>
+        <v>0.6175</v>
       </c>
       <c r="V33" t="n">
-        <v>0.36</v>
+        <v>0.3625</v>
       </c>
       <c r="W33" t="n">
         <v>0.99</v>
       </c>
       <c r="X33" t="n">
-        <v>0.62</v>
+        <v>0.6175</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.37</v>
+        <v>0.3725</v>
       </c>
       <c r="Z33" t="n">
         <v>0.99</v>
       </c>
       <c r="AA33" t="n">
-        <v>0.62</v>
+        <v>0.619</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.37</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="34">
@@ -3900,22 +3900,22 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>0.24</v>
+        <v>0.2354</v>
       </c>
       <c r="L34" t="n">
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>-0.21</v>
+        <v>-0.2146</v>
       </c>
       <c r="N34" t="n">
-        <v>0.41</v>
+        <v>0.4079</v>
       </c>
       <c r="O34" t="n">
         <v>0.47</v>
       </c>
       <c r="P34" t="n">
-        <v>-0.06</v>
+        <v>-0.0621</v>
       </c>
       <c r="Q34" t="n">
         <v>1</v>
@@ -3999,28 +3999,28 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>0.95</v>
+        <v>0.951</v>
       </c>
       <c r="M35" t="n">
-        <v>0.05</v>
+        <v>0.049</v>
       </c>
       <c r="N35" t="n">
         <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>0.95</v>
+        <v>0.954</v>
       </c>
       <c r="P35" t="n">
-        <v>0.05</v>
+        <v>0.046</v>
       </c>
       <c r="Q35" t="n">
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>0.96</v>
+        <v>0.957</v>
       </c>
       <c r="S35" t="n">
-        <v>-0.96</v>
+        <v>-0.957</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -4035,10 +4035,10 @@
         <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>0.96</v>
+        <v>0.957</v>
       </c>
       <c r="Y35" t="n">
-        <v>-0.96</v>
+        <v>-0.957</v>
       </c>
       <c r="Z35" t="n">
         <v>0.84</v>
@@ -4112,10 +4112,10 @@
         <v>0.18</v>
       </c>
       <c r="O36" t="n">
-        <v>0.34</v>
+        <v>0.335</v>
       </c>
       <c r="P36" t="n">
-        <v>-0.16</v>
+        <v>-0.155</v>
       </c>
       <c r="Q36" t="n">
         <v>0.18</v>
@@ -4130,10 +4130,10 @@
         <v>0</v>
       </c>
       <c r="U36" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="V36" t="n">
-        <v>-0.36</v>
+        <v>-0.365</v>
       </c>
       <c r="W36" t="n">
         <v>0.18</v>
@@ -4148,10 +4148,10 @@
         <v>0</v>
       </c>
       <c r="AA36" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="AB36" t="n">
-        <v>-0.36</v>
+        <v>-0.365</v>
       </c>
     </row>
     <row r="37">
@@ -4213,31 +4213,31 @@
         <v>134.62</v>
       </c>
       <c r="N37" t="n">
-        <v>0.08</v>
+        <v>0.0827</v>
       </c>
       <c r="O37" t="n">
-        <v>6.99</v>
+        <v>6.9925</v>
       </c>
       <c r="P37" t="n">
-        <v>-6.91</v>
+        <v>-6.9098</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.08</v>
+        <v>0.0827</v>
       </c>
       <c r="R37" t="n">
-        <v>6.61</v>
+        <v>6.6123</v>
       </c>
       <c r="S37" t="n">
-        <v>-6.53</v>
+        <v>-6.5296</v>
       </c>
       <c r="T37" t="n">
         <v>10.32</v>
       </c>
       <c r="U37" t="n">
-        <v>6.28</v>
+        <v>6.2823</v>
       </c>
       <c r="V37" t="n">
-        <v>4.04</v>
+        <v>4.0377</v>
       </c>
       <c r="W37" t="n">
         <v>11.1</v>

</xml_diff>